<commit_message>
Add CVS/NVO pages, notes, and DCF defaults
Add full stock coverage for CVS and NVO: new stock pages (stocks/cvs.html, stocks/nvo.html), two analysis cards in index.html, and related CSS tweaks in styles.css. Add research assets and data: new stock-note files (dividend summaries, Q4 2025 earnings transcripts, dividend analysis, trials), new Excel workbook for CVS and updated nvo.xlsx. Update documentation to set default DCF parameters (TGR 2.5%, ERP 5.5%) in .claude/equity-research/SKILL.md and CLAUDE.md. Also add a local settings command to .claude/settings.local.json to test for the generated nvo.html.
</commit_message>
<xml_diff>
--- a/excel/nvo.xlsx
+++ b/excel/nvo.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tony\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tony\Documents\GITHUB\tonynguyen22.github.io\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{74FA1E81-227E-4958-8BC4-2B2AE2AD33B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98823B7E-C255-40BF-80C9-68833730C1E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{B0FFA487-169E-4C50-9CA9-DAE968B44586}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B0FFA487-169E-4C50-9CA9-DAE968B44586}"/>
   </bookViews>
   <sheets>
     <sheet name="Income Statement" sheetId="1" r:id="rId1"/>
     <sheet name="Balance Sheet" sheetId="2" r:id="rId2"/>
     <sheet name="Cashflow" sheetId="3" r:id="rId3"/>
+    <sheet name="Ratio" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="169">
   <si>
     <t>Fiscal Year</t>
   </si>
@@ -437,13 +438,121 @@
   </si>
   <si>
     <t>Change in Working Capital</t>
+  </si>
+  <si>
+    <t>Current</t>
+  </si>
+  <si>
+    <t>Market Cap</t>
+  </si>
+  <si>
+    <t>Market Cap Growth</t>
+  </si>
+  <si>
+    <t>Enterprise Value</t>
+  </si>
+  <si>
+    <t>Last Close Price</t>
+  </si>
+  <si>
+    <t>PE Ratio</t>
+  </si>
+  <si>
+    <t>Forward PE</t>
+  </si>
+  <si>
+    <t>PS Ratio</t>
+  </si>
+  <si>
+    <t>PB Ratio</t>
+  </si>
+  <si>
+    <t>P/TBV Ratio</t>
+  </si>
+  <si>
+    <t>P/FCF Ratio</t>
+  </si>
+  <si>
+    <t>P/OCF Ratio</t>
+  </si>
+  <si>
+    <t>EV/Sales Ratio</t>
+  </si>
+  <si>
+    <t>EV/EBITDA Ratio</t>
+  </si>
+  <si>
+    <t>EV/EBIT Ratio</t>
+  </si>
+  <si>
+    <t>EV/FCF Ratio</t>
+  </si>
+  <si>
+    <t>Debt / Equity Ratio</t>
+  </si>
+  <si>
+    <t>Debt / EBITDA Ratio</t>
+  </si>
+  <si>
+    <t>Debt / FCF Ratio</t>
+  </si>
+  <si>
+    <t>Net Debt / Equity Ratio</t>
+  </si>
+  <si>
+    <t>Net Debt / EBITDA Ratio</t>
+  </si>
+  <si>
+    <t>Net Debt / FCF Ratio</t>
+  </si>
+  <si>
+    <t>Asset Turnover</t>
+  </si>
+  <si>
+    <t>Inventory Turnover</t>
+  </si>
+  <si>
+    <t>Quick Ratio</t>
+  </si>
+  <si>
+    <t>Current Ratio</t>
+  </si>
+  <si>
+    <t>Return on Equity (ROE)</t>
+  </si>
+  <si>
+    <t>Return on Assets (ROA)</t>
+  </si>
+  <si>
+    <t>Return on Invested Capital (ROIC)</t>
+  </si>
+  <si>
+    <t>Return on Capital Employed (ROCE)</t>
+  </si>
+  <si>
+    <t>Earnings Yield</t>
+  </si>
+  <si>
+    <t>FCF Yield</t>
+  </si>
+  <si>
+    <t>Dividend Yield</t>
+  </si>
+  <si>
+    <t>Payout Ratio</t>
+  </si>
+  <si>
+    <t>Buyback Yield / Dilution</t>
+  </si>
+  <si>
+    <t>Total Shareholder Return</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -485,6 +594,12 @@
     </font>
     <font>
       <b/>
+      <sz val="14"/>
+      <color rgb="FF111827"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="14"/>
       <color rgb="FF111827"/>
       <name val="Arial"/>
@@ -572,7 +687,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -639,6 +754,30 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="10" fontId="5" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3725,4 +3864,873 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FA4E4985-841C-48C4-933F-55A74A876612}">
+  <dimension ref="A1:G37"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="46.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="25" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="25" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="25" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="25" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="25" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="72.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="26">
+        <v>44561</v>
+      </c>
+      <c r="C2" s="26">
+        <v>44926</v>
+      </c>
+      <c r="D2" s="26">
+        <v>45291</v>
+      </c>
+      <c r="E2" s="26">
+        <v>45657</v>
+      </c>
+      <c r="F2" s="26">
+        <v>46022</v>
+      </c>
+      <c r="G2" s="26">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="B3" s="27">
+        <v>1664</v>
+      </c>
+      <c r="C3" s="27">
+        <v>1985</v>
+      </c>
+      <c r="D3" s="27">
+        <v>3001</v>
+      </c>
+      <c r="E3" s="27">
+        <v>2470</v>
+      </c>
+      <c r="F3" s="27">
+        <v>1461</v>
+      </c>
+      <c r="G3" s="28">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="8">
+        <v>0.57640000000000002</v>
+      </c>
+      <c r="C4" s="8">
+        <v>0.19270000000000001</v>
+      </c>
+      <c r="D4" s="8">
+        <v>0.51200000000000001</v>
+      </c>
+      <c r="E4" s="18">
+        <v>-0.17680000000000001</v>
+      </c>
+      <c r="F4" s="18">
+        <v>-0.40849999999999997</v>
+      </c>
+      <c r="G4" s="18">
+        <v>-0.54269999999999996</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="29">
+        <v>1725.97</v>
+      </c>
+      <c r="C5" s="29">
+        <v>1999.85</v>
+      </c>
+      <c r="D5" s="29">
+        <v>2972.91</v>
+      </c>
+      <c r="E5" s="29">
+        <v>2969.69</v>
+      </c>
+      <c r="F5" s="29">
+        <v>2099.91</v>
+      </c>
+      <c r="G5" s="14">
+        <v>187.15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="B6" s="30">
+        <v>56</v>
+      </c>
+      <c r="C6" s="30">
+        <v>67.67</v>
+      </c>
+      <c r="D6" s="30">
+        <v>103.45</v>
+      </c>
+      <c r="E6" s="30">
+        <v>86.02</v>
+      </c>
+      <c r="F6" s="30">
+        <v>50.88</v>
+      </c>
+      <c r="G6" s="30">
+        <v>38.58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="B7" s="14">
+        <v>35.31</v>
+      </c>
+      <c r="C7" s="14">
+        <v>38.47</v>
+      </c>
+      <c r="D7" s="14">
+        <v>37.53</v>
+      </c>
+      <c r="E7" s="14">
+        <v>27.24</v>
+      </c>
+      <c r="F7" s="14">
+        <v>14.06</v>
+      </c>
+      <c r="G7" s="14">
+        <v>10.62</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8" s="14">
+        <v>11.82</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="B9" s="14">
+        <v>1.84</v>
+      </c>
+      <c r="C9" s="14">
+        <v>1.74</v>
+      </c>
+      <c r="D9" s="14">
+        <v>2.0099999999999998</v>
+      </c>
+      <c r="E9" s="14">
+        <v>1.32</v>
+      </c>
+      <c r="F9" s="14">
+        <v>0.74</v>
+      </c>
+      <c r="G9" s="14">
+        <v>3.52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="B10" s="14">
+        <v>3.66</v>
+      </c>
+      <c r="C10" s="14">
+        <v>3.7</v>
+      </c>
+      <c r="D10" s="14">
+        <v>4.38</v>
+      </c>
+      <c r="E10" s="14">
+        <v>2.68</v>
+      </c>
+      <c r="F10" s="14">
+        <v>1.17</v>
+      </c>
+      <c r="G10" s="14">
+        <v>5.61</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="B11" s="14">
+        <v>3.65</v>
+      </c>
+      <c r="C11" s="14">
+        <v>3.68</v>
+      </c>
+      <c r="D11" s="14">
+        <v>4.3600000000000003</v>
+      </c>
+      <c r="E11" s="14">
+        <v>2.68</v>
+      </c>
+      <c r="F11" s="14">
+        <v>1.17</v>
+      </c>
+      <c r="G11" s="14">
+        <v>0.88</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="B12" s="14">
+        <v>5.32</v>
+      </c>
+      <c r="C12" s="14">
+        <v>4.62</v>
+      </c>
+      <c r="D12" s="14">
+        <v>5.61</v>
+      </c>
+      <c r="E12" s="14">
+        <v>5.2</v>
+      </c>
+      <c r="F12" s="14">
+        <v>3.85</v>
+      </c>
+      <c r="G12" s="14">
+        <v>18.649999999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="B13" s="14">
+        <v>4.7</v>
+      </c>
+      <c r="C13" s="14">
+        <v>3.91</v>
+      </c>
+      <c r="D13" s="14">
+        <v>4.28</v>
+      </c>
+      <c r="E13" s="14">
+        <v>3.18</v>
+      </c>
+      <c r="F13" s="14">
+        <v>1.91</v>
+      </c>
+      <c r="G13" s="14">
+        <v>9.1300000000000008</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="B14" s="14">
+        <v>1.91</v>
+      </c>
+      <c r="C14" s="14">
+        <v>1.76</v>
+      </c>
+      <c r="D14" s="14">
+        <v>1.99</v>
+      </c>
+      <c r="E14" s="14">
+        <v>1.59</v>
+      </c>
+      <c r="F14" s="14">
+        <v>1.06</v>
+      </c>
+      <c r="G14" s="14">
+        <v>3.85</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="B15" s="14">
+        <v>4.1500000000000004</v>
+      </c>
+      <c r="C15" s="14">
+        <v>3.78</v>
+      </c>
+      <c r="D15" s="14">
+        <v>4.13</v>
+      </c>
+      <c r="E15" s="14">
+        <v>3.13</v>
+      </c>
+      <c r="F15" s="14">
+        <v>2.1800000000000002</v>
+      </c>
+      <c r="G15" s="14">
+        <v>7.77</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B16" s="14">
+        <v>4.58</v>
+      </c>
+      <c r="C16" s="14">
+        <v>4.16</v>
+      </c>
+      <c r="D16" s="14">
+        <v>4.51</v>
+      </c>
+      <c r="E16" s="14">
+        <v>3.6</v>
+      </c>
+      <c r="F16" s="14">
+        <v>2.56</v>
+      </c>
+      <c r="G16" s="14">
+        <v>8.4700000000000006</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="B17" s="30">
+        <v>5.51</v>
+      </c>
+      <c r="C17" s="30">
+        <v>4.66</v>
+      </c>
+      <c r="D17" s="30">
+        <v>5.56</v>
+      </c>
+      <c r="E17" s="30">
+        <v>6.26</v>
+      </c>
+      <c r="F17" s="30">
+        <v>5.54</v>
+      </c>
+      <c r="G17" s="30">
+        <v>20.41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="B18" s="14">
+        <v>0.41</v>
+      </c>
+      <c r="C18" s="14">
+        <v>0.34</v>
+      </c>
+      <c r="D18" s="14">
+        <v>0.27</v>
+      </c>
+      <c r="E18" s="14">
+        <v>0.77</v>
+      </c>
+      <c r="F18" s="14">
+        <v>0.69</v>
+      </c>
+      <c r="G18" s="14">
+        <v>0.69</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="B19" s="14">
+        <v>0.45</v>
+      </c>
+      <c r="C19" s="14">
+        <v>0.35</v>
+      </c>
+      <c r="D19" s="14">
+        <v>0.25</v>
+      </c>
+      <c r="E19" s="14">
+        <v>0.75</v>
+      </c>
+      <c r="F19" s="14">
+        <v>0.89</v>
+      </c>
+      <c r="G19" s="14">
+        <v>0.89</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="B20" s="14">
+        <v>0.59</v>
+      </c>
+      <c r="C20" s="14">
+        <v>0.43</v>
+      </c>
+      <c r="D20" s="14">
+        <v>0.34</v>
+      </c>
+      <c r="E20" s="14">
+        <v>1.5</v>
+      </c>
+      <c r="F20" s="14">
+        <v>2.2599999999999998</v>
+      </c>
+      <c r="G20" s="14">
+        <v>2.2599999999999998</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="B21" s="14">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="C21" s="14">
+        <v>0.03</v>
+      </c>
+      <c r="D21" s="14">
+        <v>-0.04</v>
+      </c>
+      <c r="E21" s="14">
+        <v>0.54</v>
+      </c>
+      <c r="F21" s="14">
+        <v>0.51</v>
+      </c>
+      <c r="G21" s="14">
+        <v>0.51</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="B22" s="14">
+        <v>0.15</v>
+      </c>
+      <c r="C22" s="14">
+        <v>0.03</v>
+      </c>
+      <c r="D22" s="14">
+        <v>-0.04</v>
+      </c>
+      <c r="E22" s="14">
+        <v>0.53</v>
+      </c>
+      <c r="F22" s="14">
+        <v>0.66</v>
+      </c>
+      <c r="G22" s="14">
+        <v>0.66</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="B23" s="30">
+        <v>0.2</v>
+      </c>
+      <c r="C23" s="30">
+        <v>0.04</v>
+      </c>
+      <c r="D23" s="30">
+        <v>-0.05</v>
+      </c>
+      <c r="E23" s="30">
+        <v>1.05</v>
+      </c>
+      <c r="F23" s="30">
+        <v>1.69</v>
+      </c>
+      <c r="G23" s="30">
+        <v>1.69</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="B24" s="14">
+        <v>0.83</v>
+      </c>
+      <c r="C24" s="14">
+        <v>0.81</v>
+      </c>
+      <c r="D24" s="14">
+        <v>0.84</v>
+      </c>
+      <c r="E24" s="14">
+        <v>0.74</v>
+      </c>
+      <c r="F24" s="14">
+        <v>0.61</v>
+      </c>
+      <c r="G24" s="14">
+        <v>0.61</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="B25" s="14">
+        <v>1.24</v>
+      </c>
+      <c r="C25" s="14">
+        <v>1.29</v>
+      </c>
+      <c r="D25" s="14">
+        <v>1.27</v>
+      </c>
+      <c r="E25" s="14">
+        <v>1.23</v>
+      </c>
+      <c r="F25" s="14">
+        <v>1.3</v>
+      </c>
+      <c r="G25" s="14">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="B26" s="14">
+        <v>0.67</v>
+      </c>
+      <c r="C26" s="14">
+        <v>0.69</v>
+      </c>
+      <c r="D26" s="14">
+        <v>0.64</v>
+      </c>
+      <c r="E26" s="14">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="F26" s="14">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="G26" s="14">
+        <v>0.56999999999999995</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="B27" s="30">
+        <v>0.86</v>
+      </c>
+      <c r="C27" s="30">
+        <v>0.89</v>
+      </c>
+      <c r="D27" s="30">
+        <v>0.82</v>
+      </c>
+      <c r="E27" s="30">
+        <v>0.74</v>
+      </c>
+      <c r="F27" s="30">
+        <v>0.8</v>
+      </c>
+      <c r="G27" s="30">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="B28" s="31">
+        <v>0.71240000000000003</v>
+      </c>
+      <c r="C28" s="31">
+        <v>0.72</v>
+      </c>
+      <c r="D28" s="31">
+        <v>0.88070000000000004</v>
+      </c>
+      <c r="E28" s="31">
+        <v>0.80779999999999996</v>
+      </c>
+      <c r="F28" s="31">
+        <v>0.60699999999999998</v>
+      </c>
+      <c r="G28" s="31">
+        <v>0.60699999999999998</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="B29" s="31">
+        <v>0.27929999999999999</v>
+      </c>
+      <c r="C29" s="31">
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="D29" s="31">
+        <v>0.29509999999999997</v>
+      </c>
+      <c r="E29" s="31">
+        <v>0.26119999999999999</v>
+      </c>
+      <c r="F29" s="31">
+        <v>0.1986</v>
+      </c>
+      <c r="G29" s="31">
+        <v>0.1986</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="B30" s="31">
+        <v>0.37380000000000002</v>
+      </c>
+      <c r="C30" s="31">
+        <v>0.37340000000000001</v>
+      </c>
+      <c r="D30" s="31">
+        <v>0.40689999999999998</v>
+      </c>
+      <c r="E30" s="31">
+        <v>0.34329999999999999</v>
+      </c>
+      <c r="F30" s="31">
+        <v>0.2455</v>
+      </c>
+      <c r="G30" s="31">
+        <v>0.2455</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="B31" s="31">
+        <v>0.69140000000000001</v>
+      </c>
+      <c r="C31" s="31">
+        <v>0.69489999999999996</v>
+      </c>
+      <c r="D31" s="31">
+        <v>0.77370000000000005</v>
+      </c>
+      <c r="E31" s="31">
+        <v>0.65300000000000002</v>
+      </c>
+      <c r="F31" s="31">
+        <v>0.44359999999999999</v>
+      </c>
+      <c r="G31" s="31">
+        <v>0.44359999999999999</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="B32" s="31">
+        <v>2.8299999999999999E-2</v>
+      </c>
+      <c r="C32" s="31">
+        <v>2.5999999999999999E-2</v>
+      </c>
+      <c r="D32" s="31">
+        <v>2.6599999999999999E-2</v>
+      </c>
+      <c r="E32" s="31">
+        <v>3.6700000000000003E-2</v>
+      </c>
+      <c r="F32" s="31">
+        <v>7.1099999999999997E-2</v>
+      </c>
+      <c r="G32" s="31">
+        <v>9.4200000000000006E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="B33" s="31">
+        <v>0.18809999999999999</v>
+      </c>
+      <c r="C33" s="31">
+        <v>0.21629999999999999</v>
+      </c>
+      <c r="D33" s="31">
+        <v>0.17810000000000001</v>
+      </c>
+      <c r="E33" s="31">
+        <v>0.19220000000000001</v>
+      </c>
+      <c r="F33" s="31">
+        <v>0.25950000000000001</v>
+      </c>
+      <c r="G33" s="31">
+        <v>5.3600000000000002E-2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="B34" s="31">
+        <v>1.2800000000000001E-2</v>
+      </c>
+      <c r="C34" s="31">
+        <v>1.1900000000000001E-2</v>
+      </c>
+      <c r="D34" s="31">
+        <v>1.01E-2</v>
+      </c>
+      <c r="E34" s="31">
+        <v>1.61E-2</v>
+      </c>
+      <c r="F34" s="31">
+        <v>3.5900000000000001E-2</v>
+      </c>
+      <c r="G34" s="31">
+        <v>3.1899999999999998E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="B35" s="31">
+        <v>0.4506</v>
+      </c>
+      <c r="C35" s="31">
+        <v>0.45569999999999999</v>
+      </c>
+      <c r="D35" s="31">
+        <v>0.37959999999999999</v>
+      </c>
+      <c r="E35" s="31">
+        <v>0.43709999999999999</v>
+      </c>
+      <c r="F35" s="31">
+        <v>0.50529999999999997</v>
+      </c>
+      <c r="G35" s="31">
+        <v>0.33989999999999998</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="18.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="B36" s="31">
+        <v>7.5200000000000003E-2</v>
+      </c>
+      <c r="C36" s="31">
+        <v>7.8100000000000003E-2</v>
+      </c>
+      <c r="D36" s="31">
+        <v>6.4100000000000004E-2</v>
+      </c>
+      <c r="E36" s="31">
+        <v>5.2499999999999998E-2</v>
+      </c>
+      <c r="F36" s="31">
+        <v>6.1000000000000004E-3</v>
+      </c>
+      <c r="G36" s="31">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+      <c r="A37" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="B37" s="31">
+        <v>8.7999999999999995E-2</v>
+      </c>
+      <c r="C37" s="31">
+        <v>8.9899999999999994E-2</v>
+      </c>
+      <c r="D37" s="31">
+        <v>7.4300000000000005E-2</v>
+      </c>
+      <c r="E37" s="31">
+        <v>6.8599999999999994E-2</v>
+      </c>
+      <c r="F37" s="31">
+        <v>4.2000000000000003E-2</v>
+      </c>
+      <c r="G37" s="31">
+        <v>3.2899999999999999E-2</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A3" r:id="rId1" display="https://stockanalysis.com/stocks/nvo/market-cap/" xr:uid="{77F89371-9A0C-4729-B78D-D08E14DE0E06}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>